<commit_message>
Removing year from wind onshore's availability factor per timestamp
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_EE_SubAnnualData.xlsx
+++ b/SuppXLS/Scen_EE_SubAnnualData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F79DEA0-8B1E-4CDE-A8D7-CAB91FC1D297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CCB1F04-08D9-47BF-BA33-FDCCBDF196CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="33">
   <si>
     <t>S01aH01</t>
   </si>
@@ -120,9 +120,6 @@
   </si>
   <si>
     <t>LimType</t>
-  </si>
-  <si>
-    <t>Year</t>
   </si>
   <si>
     <t>Pset_PN</t>
@@ -501,13 +498,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:G28"/>
+  <dimension ref="B3:F28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>24</v>
       </c>
@@ -515,9 +512,8 @@
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>25</v>
       </c>
@@ -527,494 +523,419 @@
       <c r="D4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E5">
-        <v>2025</v>
-      </c>
-      <c r="F5">
         <v>0.30733467260353509</v>
       </c>
-      <c r="G5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E6">
-        <v>2025</v>
-      </c>
-      <c r="F6">
         <v>0.31081408677879568</v>
       </c>
-      <c r="G6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E7">
-        <v>2025</v>
-      </c>
-      <c r="F7">
         <v>0.28004877849483201</v>
       </c>
-      <c r="G7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E8">
-        <v>2025</v>
-      </c>
-      <c r="F8">
         <v>0.28531085095827602</v>
       </c>
-      <c r="G8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>4</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E9">
-        <v>2025</v>
-      </c>
-      <c r="F9">
         <v>0.32854279458298841</v>
       </c>
-      <c r="G9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E10">
-        <v>2025</v>
-      </c>
-      <c r="F10">
         <v>0.31788704311118388</v>
       </c>
-      <c r="G10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E11">
-        <v>2025</v>
-      </c>
-      <c r="F11">
         <v>0.23562337842422371</v>
       </c>
-      <c r="G11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E12">
-        <v>2025</v>
-      </c>
-      <c r="F12">
         <v>0.18514551916650079</v>
       </c>
-      <c r="G12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E13">
-        <v>2025</v>
-      </c>
-      <c r="F13">
         <v>0.1792466671197426</v>
       </c>
-      <c r="G13" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>9</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E14">
-        <v>2025</v>
-      </c>
-      <c r="F14">
         <v>0.18502434111283389</v>
       </c>
-      <c r="G14" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E15">
-        <v>2025</v>
-      </c>
-      <c r="F15">
         <v>0.21110444202613651</v>
       </c>
-      <c r="G15" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>11</v>
       </c>
       <c r="C16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E16">
-        <v>2025</v>
-      </c>
-      <c r="F16">
         <v>0.24879047443284069</v>
       </c>
-      <c r="G16" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F16" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E17">
-        <v>2025</v>
-      </c>
-      <c r="F17">
         <v>0.1463192433507913</v>
       </c>
-      <c r="G17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E18">
-        <v>2025</v>
-      </c>
-      <c r="F18">
         <v>0.12774788307594531</v>
       </c>
-      <c r="G18" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E19">
-        <v>2025</v>
-      </c>
-      <c r="F19">
         <v>0.1411084812546918</v>
       </c>
-      <c r="G19" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>15</v>
       </c>
       <c r="C20" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E20">
-        <v>2025</v>
-      </c>
-      <c r="F20">
         <v>0.14456244232963339</v>
       </c>
-      <c r="G20" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E21">
-        <v>2025</v>
-      </c>
-      <c r="F21">
         <v>0.15290090042974089</v>
       </c>
-      <c r="G21" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>17</v>
       </c>
       <c r="C22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E22">
-        <v>2025</v>
-      </c>
-      <c r="F22">
         <v>0.15616170136503871</v>
       </c>
-      <c r="G22" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>18</v>
       </c>
       <c r="C23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E23">
-        <v>2025</v>
-      </c>
-      <c r="F23">
         <v>0.2711239713139022</v>
       </c>
-      <c r="G23" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F23" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>19</v>
       </c>
       <c r="C24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E24">
-        <v>2025</v>
-      </c>
-      <c r="F24">
         <v>0.25541442832837402</v>
       </c>
-      <c r="G24" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F24" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>20</v>
       </c>
       <c r="C25" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E25">
-        <v>2025</v>
-      </c>
-      <c r="F25">
         <v>0.24428965887155499</v>
       </c>
-      <c r="G25" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F25" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>21</v>
       </c>
       <c r="C26" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E26">
-        <v>2025</v>
-      </c>
-      <c r="F26">
         <v>0.25342572224556742</v>
       </c>
-      <c r="G26" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F26" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>22</v>
       </c>
       <c r="C27" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E27">
-        <v>2025</v>
-      </c>
-      <c r="F27">
         <v>0.29266764618764368</v>
       </c>
-      <c r="G27" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>23</v>
       </c>
       <c r="C28" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D28" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E28">
-        <v>2025</v>
-      </c>
-      <c r="F28">
         <v>0.29668217122661111</v>
       </c>
-      <c r="G28" t="s">
-        <v>33</v>
+      <c r="F28" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
attempt on fixing timeslice issue with windon
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_EE_SubAnnualData.xlsx
+++ b/SuppXLS/Scen_EE_SubAnnualData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CCB1F04-08D9-47BF-BA33-FDCCBDF196CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC3A3CB1-976B-46C0-98C8-6D6FEDE1EEDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Windon" sheetId="1" r:id="rId1"/>
@@ -38,78 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="33">
   <si>
-    <t>S01aH01</t>
-  </si>
-  <si>
-    <t>S01aH02</t>
-  </si>
-  <si>
-    <t>S01aH03</t>
-  </si>
-  <si>
-    <t>S01aH04</t>
-  </si>
-  <si>
-    <t>S01aH05</t>
-  </si>
-  <si>
-    <t>S01aH06</t>
-  </si>
-  <si>
-    <t>S02aH01</t>
-  </si>
-  <si>
-    <t>S02aH02</t>
-  </si>
-  <si>
-    <t>S02aH03</t>
-  </si>
-  <si>
-    <t>S02aH04</t>
-  </si>
-  <si>
-    <t>S02aH05</t>
-  </si>
-  <si>
-    <t>S02aH06</t>
-  </si>
-  <si>
-    <t>S03aH01</t>
-  </si>
-  <si>
-    <t>S03aH02</t>
-  </si>
-  <si>
-    <t>S03aH03</t>
-  </si>
-  <si>
-    <t>S03aH04</t>
-  </si>
-  <si>
-    <t>S03aH05</t>
-  </si>
-  <si>
-    <t>S03aH06</t>
-  </si>
-  <si>
-    <t>S04aH01</t>
-  </si>
-  <si>
-    <t>S04aH02</t>
-  </si>
-  <si>
-    <t>S04aH03</t>
-  </si>
-  <si>
-    <t>S04aH04</t>
-  </si>
-  <si>
-    <t>S04aH05</t>
-  </si>
-  <si>
-    <t>S04aH06</t>
-  </si>
-  <si>
     <t>~TFM_DINS</t>
   </si>
   <si>
@@ -135,6 +63,78 @@
   </si>
   <si>
     <t>ELEWON</t>
+  </si>
+  <si>
+    <t>S01H02</t>
+  </si>
+  <si>
+    <t>S01H03</t>
+  </si>
+  <si>
+    <t>S01H04</t>
+  </si>
+  <si>
+    <t>S01H05</t>
+  </si>
+  <si>
+    <t>S01H06</t>
+  </si>
+  <si>
+    <t>S02H01</t>
+  </si>
+  <si>
+    <t>S02H02</t>
+  </si>
+  <si>
+    <t>S02H03</t>
+  </si>
+  <si>
+    <t>S02H04</t>
+  </si>
+  <si>
+    <t>S02H05</t>
+  </si>
+  <si>
+    <t>S02H06</t>
+  </si>
+  <si>
+    <t>S03H01</t>
+  </si>
+  <si>
+    <t>S03H02</t>
+  </si>
+  <si>
+    <t>S03H03</t>
+  </si>
+  <si>
+    <t>S03H04</t>
+  </si>
+  <si>
+    <t>S03H05</t>
+  </si>
+  <si>
+    <t>S03H06</t>
+  </si>
+  <si>
+    <t>S04H01</t>
+  </si>
+  <si>
+    <t>S04H02</t>
+  </si>
+  <si>
+    <t>S04H03</t>
+  </si>
+  <si>
+    <t>S04H04</t>
+  </si>
+  <si>
+    <t>S04H05</t>
+  </si>
+  <si>
+    <t>S04H06</t>
+  </si>
+  <si>
+    <t>S01H01</t>
   </si>
 </sst>
 </file>
@@ -506,7 +506,7 @@
   <sheetData>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -515,427 +515,427 @@
     </row>
     <row r="4" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>28</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E5">
         <v>0.30733467260353509</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E6">
         <v>0.31081408677879568</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E7">
         <v>0.28004877849483201</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E8">
         <v>0.28531085095827602</v>
       </c>
       <c r="F8" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E9">
         <v>0.32854279458298841</v>
       </c>
       <c r="F9" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D10" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E10">
         <v>0.31788704311118388</v>
       </c>
       <c r="F10" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E11">
         <v>0.23562337842422371</v>
       </c>
       <c r="F11" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E12">
         <v>0.18514551916650079</v>
       </c>
       <c r="F12" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D13" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E13">
         <v>0.1792466671197426</v>
       </c>
       <c r="F13" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E14">
         <v>0.18502434111283389</v>
       </c>
       <c r="F14" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E15">
         <v>0.21110444202613651</v>
       </c>
       <c r="F15" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C16" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D16" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E16">
         <v>0.24879047443284069</v>
       </c>
       <c r="F16" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C17" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D17" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E17">
         <v>0.1463192433507913</v>
       </c>
       <c r="F17" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C18" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E18">
         <v>0.12774788307594531</v>
       </c>
       <c r="F18" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C19" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D19" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E19">
         <v>0.1411084812546918</v>
       </c>
       <c r="F19" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D20" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E20">
         <v>0.14456244232963339</v>
       </c>
       <c r="F20" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E21">
         <v>0.15290090042974089</v>
       </c>
       <c r="F21" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D22" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E22">
         <v>0.15616170136503871</v>
       </c>
       <c r="F22" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D23" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E23">
         <v>0.2711239713139022</v>
       </c>
       <c r="F23" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C24" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D24" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E24">
         <v>0.25541442832837402</v>
       </c>
       <c r="F24" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C25" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D25" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E25">
         <v>0.24428965887155499</v>
       </c>
       <c r="F25" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C26" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D26" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E26">
         <v>0.25342572224556742</v>
       </c>
       <c r="F26" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C27" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D27" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E27">
         <v>0.29266764618764368</v>
       </c>
       <c r="F27" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C28" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="D28" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E28">
         <v>0.29668217122661111</v>
       </c>
       <c r="F28" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding availability factor to PV
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_EE_SubAnnualData.xlsx
+++ b/SuppXLS/Scen_EE_SubAnnualData.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D200F3-EE51-411E-8758-092BA8C9FE76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B5980F1-BDD2-46A4-8EB2-AFEEA6626674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Windon" sheetId="1" r:id="rId1"/>
+    <sheet name="PV" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -71,8 +72,44 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Kristopher Raik</author>
+  </authors>
+  <commentList>
+    <comment ref="B3" authorId="0" shapeId="0" xr:uid="{543EBC6D-7463-4399-A6EC-DC78C12233E3}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="186"/>
+          </rPr>
+          <t>Kristopher Raik:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+            <charset val="186"/>
+          </rPr>
+          <t xml:space="preserve">
+DINS?</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="34">
   <si>
     <t>TimeSlice</t>
   </si>
@@ -171,6 +208,9 @@
   </si>
   <si>
     <t>~TFM_INS</t>
+  </si>
+  <si>
+    <t>ELESOL</t>
   </si>
 </sst>
 </file>
@@ -994,4 +1034,449 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3480837-D79F-4A83-9EB5-08D62B96490A}">
+  <dimension ref="B3:F28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>1.6646321763888888E-2</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>0.1709819009777778</v>
+      </c>
+      <c r="F7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8">
+        <v>0.12684142476944441</v>
+      </c>
+      <c r="F8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>2.7973095972222222E-3</v>
+      </c>
+      <c r="F9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11">
+        <v>3.0382599384615378E-3</v>
+      </c>
+      <c r="F11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" t="s">
+        <v>4</v>
+      </c>
+      <c r="E12">
+        <v>0.15561345699175819</v>
+      </c>
+      <c r="F12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13">
+        <v>0.43306220051098898</v>
+      </c>
+      <c r="F13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" t="s">
+        <v>4</v>
+      </c>
+      <c r="E14">
+        <v>0.34494600395879121</v>
+      </c>
+      <c r="F14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15">
+        <v>5.361769763461538E-2</v>
+      </c>
+      <c r="F15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16">
+        <v>1.2226972527472529E-5</v>
+      </c>
+      <c r="F16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" t="s">
+        <v>4</v>
+      </c>
+      <c r="E17">
+        <v>1.4058011809782609E-3</v>
+      </c>
+      <c r="F17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" t="s">
+        <v>3</v>
+      </c>
+      <c r="D18" t="s">
+        <v>4</v>
+      </c>
+      <c r="E18">
+        <v>0.11990599222282609</v>
+      </c>
+      <c r="F18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>4</v>
+      </c>
+      <c r="E19">
+        <v>0.37081215739402168</v>
+      </c>
+      <c r="F19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" t="s">
+        <v>4</v>
+      </c>
+      <c r="E20">
+        <v>0.28381095157065223</v>
+      </c>
+      <c r="F20" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" t="s">
+        <v>3</v>
+      </c>
+      <c r="D21" t="s">
+        <v>4</v>
+      </c>
+      <c r="E21">
+        <v>3.9219056866847818E-2</v>
+      </c>
+      <c r="F21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" t="s">
+        <v>4</v>
+      </c>
+      <c r="E22">
+        <v>1.6792282608695651E-6</v>
+      </c>
+      <c r="F22" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D23" t="s">
+        <v>4</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" t="s">
+        <v>3</v>
+      </c>
+      <c r="D24" t="s">
+        <v>4</v>
+      </c>
+      <c r="E24">
+        <v>8.2955046222826095E-3</v>
+      </c>
+      <c r="F24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" t="s">
+        <v>3</v>
+      </c>
+      <c r="D25" t="s">
+        <v>4</v>
+      </c>
+      <c r="E25">
+        <v>0.1207430217092391</v>
+      </c>
+      <c r="F25" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" t="s">
+        <v>3</v>
+      </c>
+      <c r="D26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E26">
+        <v>6.4467875070652172E-2</v>
+      </c>
+      <c r="F26" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27" t="s">
+        <v>4</v>
+      </c>
+      <c r="E27">
+        <v>1.219597608695652E-4</v>
+      </c>
+      <c r="F27" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" t="s">
+        <v>3</v>
+      </c>
+      <c r="D28" t="s">
+        <v>4</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>